<commit_message>
feat(narrative): update dialogue and settings UI
</commit_message>
<xml_diff>
--- a/GameConfig/Datas/叙事Session配置表.xlsx
+++ b/GameConfig/Datas/叙事Session配置表.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,11 @@
           <t>isFormalEnding</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>npcSet</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +514,11 @@
           <t>bool</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -556,6 +566,11 @@
           <t>是否在日终后进入正式结局</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>按剧情配表 Session.NPCSet 的顺序填写 NPC 名，逗号分隔；用于 NPC 对话左右站位</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,6 +618,11 @@
           <t>c</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -639,6 +659,11 @@
       <c r="I5" t="b">
         <v>0</v>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>老周,陈先生</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -669,11 +694,19 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>我能理解钟表的构造，却无法解释老周为何记得这次失约。若我记住了他的遗憾，这算不算也开始理解？</t>
+          <t>2026年10月6日，第24次启动。
+今日检测物品：老式座钟×1
+检测结果：达到【低效物】标准，但物主对其有强烈【情感】寄托，不建议直接按【低效物】处理标准处理，交由物主本人判断。
+钟里……有很多以前的故事，明明隔了那么久，却感觉还是那么鲜活。</t>
         </is>
       </c>
       <c r="I6" t="b">
         <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>老周</t>
+        </is>
       </c>
     </row>
     <row r="7">

</xml_diff>